<commit_message>
add Database3 (Winter Bird Survey) cleaning pipeline
Add 6-step cleaning pipeline for Winter Bird Survey data (2013-2015).
Includes extraction, ID assignment, geography validation, required
field checks, column selection, deduplication, and final report
generation. Output files for years 2013-2015 included.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3/Winter Birds '13.xlsx
+++ b/Databases/Database3/Winter Birds '13.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohanpoudel/Documents/USFWS/PipingPlover/Databases/Database3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13E39FB-C2F2-1447-96F9-D984F4D3392E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0A642F-607E-8246-B1FC-5F6AF46FAF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14640" yWindow="-21000" windowWidth="19200" windowHeight="21000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4560" yWindow="-21000" windowWidth="19200" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1632" uniqueCount="882">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1633" uniqueCount="882">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -3359,6 +3359,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="38" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="9" t="s">
+        <v>875</v>
+      </c>
       <c r="F1" s="9" t="s">
         <v>875</v>
       </c>

</xml_diff>